<commit_message>
Add the refund reason columns to the delivered disbursement upload template and refresh the template README
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VKNMX59m598zKXcFetnd5X
</commit_message>
<xml_diff>
--- a/docs/package/05_Delivery/Upload_Templates/Disbursements_Upload_Template.xlsx
+++ b/docs/package/05_Delivery/Upload_Templates/Disbursements_Upload_Template.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="81">
   <si>
     <t xml:space="preserve">Voucher Date</t>
   </si>
@@ -48,6 +48,12 @@
     <t xml:space="preserve">Remarks</t>
   </si>
   <si>
+    <t xml:space="preserve">Refund Reason</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refund Note</t>
+  </si>
+  <si>
     <t xml:space="preserve">2026-10-06</t>
   </si>
   <si>
@@ -166,6 +172,18 @@
   </si>
   <si>
     <t xml:space="preserve">remarks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer refund: reason code of the refund context (e.g. REF-CANCEL); required with disbursements.refund_reason_required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">refundReasonCode, refundReason</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note of the refund reason, when the reason asks for one</t>
+  </si>
+  <si>
+    <t xml:space="preserve">refundNote</t>
   </si>
   <si>
     <t xml:space="preserve">Item</t>
@@ -425,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -439,9 +457,11 @@
     <col min="9" max="9" width="22" customWidth="1"/>
     <col min="10" max="10" width="29" customWidth="1"/>
     <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="12" width="19" customWidth="1"/>
+    <col min="13" max="13" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="20" customHeight="1">
+    <row r="1" spans="1:13" ht="20" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -475,31 +495,37 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K2" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -509,7 +535,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -522,22 +548,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="20" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2">
@@ -545,16 +571,16 @@
         <v>0</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3">
@@ -562,19 +588,19 @@
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4">
@@ -582,13 +608,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5">
@@ -596,16 +622,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
@@ -613,16 +639,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7">
@@ -630,13 +656,13 @@
         <v>5</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8">
@@ -644,16 +670,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9">
@@ -661,16 +687,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10">
@@ -678,13 +704,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11">
@@ -692,16 +718,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12">
@@ -709,16 +735,44 @@
         <v>10</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -737,98 +791,98 @@
   <sheetData>
     <row r="1" spans="1:2" ht="20" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>